<commit_message>
Update example input file, remove redundant comments in `scheduler.cpp`, and modify related resources.
</commit_message>
<xml_diff>
--- a/SolucionesAMano.xlsx
+++ b/SolucionesAMano.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\SO\SchedulingSimSO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{453F1BDA-A594-4261-BD65-FF98B9BBDCB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D393F627-FCC4-4A20-8A6A-025AD7C83C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{11B297BD-CEE9-43C0-9F75-E94FA468A999}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="74">
   <si>
     <t>Etiqueta</t>
   </si>
@@ -189,12 +189,6 @@
     <t>31-32</t>
   </si>
   <si>
-    <t>.\SchedulingSimSO.exe ejem1.txt MLFQ 4 1 3 4 SJF</t>
-  </si>
-  <si>
-    <t>.\SchedulingSimSO.exe ejem2.txt MLFQ 4 2 3 4 PSJF</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
@@ -205,13 +199,73 @@
   </si>
   <si>
     <t>Q4</t>
+  </si>
+  <si>
+    <t>0-3</t>
+  </si>
+  <si>
+    <t>3-6</t>
+  </si>
+  <si>
+    <t>6-9</t>
+  </si>
+  <si>
+    <t>9-12</t>
+  </si>
+  <si>
+    <t>12-15</t>
+  </si>
+  <si>
+    <t>15-20</t>
+  </si>
+  <si>
+    <t>20-25</t>
+  </si>
+  <si>
+    <t>25-30</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>30-35</t>
+  </si>
+  <si>
+    <t>35-36</t>
+  </si>
+  <si>
+    <t>36-37</t>
+  </si>
+  <si>
+    <t>37-42</t>
+  </si>
+  <si>
+    <t>42-45</t>
+  </si>
+  <si>
+    <t>45-50</t>
+  </si>
+  <si>
+    <t>50-54</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,13 +279,50 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -243,22 +334,41 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -287,7 +397,7 @@
     <tableColumn id="3" xr3:uid="{CDD6AA90-A20C-42A9-A11C-01B31338C78B}" name="AT"/>
     <tableColumn id="4" xr3:uid="{4CAE9473-2C7D-4991-A9DF-F94269CA43DB}" name="Q"/>
     <tableColumn id="5" xr3:uid="{60DB5986-4F47-4AB9-B357-B903E2067D7D}" name="PR"/>
-    <tableColumn id="6" xr3:uid="{05D3CD1F-65B9-433A-9B27-FF81CEB8E7F8}" name="WT" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{05D3CD1F-65B9-433A-9B27-FF81CEB8E7F8}" name="WT" dataDxfId="2">
       <calculatedColumnFormula>4+11</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{2FBF0539-86A4-418A-B71E-C57038920F5A}" name="CT"/>
@@ -307,12 +417,32 @@
     <tableColumn id="3" xr3:uid="{7A73770F-8B76-4DB0-BE8A-7BD51690F63E}" name="AT"/>
     <tableColumn id="4" xr3:uid="{EE8BE04A-CA58-47ED-8B7B-EA16674BFED6}" name="Q"/>
     <tableColumn id="5" xr3:uid="{E32FB483-1BE3-4D58-8FA7-57B6EE2045C7}" name="PR"/>
-    <tableColumn id="6" xr3:uid="{5F6FAC81-092E-45E2-8ED6-622AE83E1BF8}" name="WT" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{5F6FAC81-092E-45E2-8ED6-622AE83E1BF8}" name="WT" dataDxfId="1">
       <calculatedColumnFormula>4+11</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{1308CF1D-E739-47B4-ACD0-5593B50FAE26}" name="CT"/>
     <tableColumn id="8" xr3:uid="{1D888F5A-680B-40DC-A733-8B020E4A418F}" name="RT"/>
     <tableColumn id="9" xr3:uid="{B87A6A09-DE1D-49EE-BE05-C8C9BE060C74}" name="TAT"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7B05F858-749A-415F-BDB8-73E05592B886}" name="Tabla134" displayName="Tabla134" ref="D43:L49" totalsRowShown="0">
+  <autoFilter ref="D43:L49" xr:uid="{7B05F858-749A-415F-BDB8-73E05592B886}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{C4D08DF5-44B4-4129-8B05-A2998620A23D}" name="Etiqueta"/>
+    <tableColumn id="2" xr3:uid="{B62E7C8C-734D-4BD9-82A0-97F045936E1A}" name="BT"/>
+    <tableColumn id="3" xr3:uid="{81EE1B97-5A7A-464D-9E6A-29007667E5BD}" name="AT"/>
+    <tableColumn id="4" xr3:uid="{38FBF5E4-6D6A-4840-A65A-EE55F7C4A0C9}" name="Q"/>
+    <tableColumn id="5" xr3:uid="{1764FD0B-C6E2-49E6-B6C9-AD91BFD81D97}" name="PR"/>
+    <tableColumn id="6" xr3:uid="{ACDA8567-AAD4-425F-8E47-C3B7BC87AA76}" name="WT" dataDxfId="0">
+      <calculatedColumnFormula>4+11</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{057B5C8B-0F1B-4CDF-A5D0-D2FA0FB23B06}" name="CT"/>
+    <tableColumn id="8" xr3:uid="{CCB545F2-F1F1-46AB-8FC7-5A212531B1B7}" name="RT"/>
+    <tableColumn id="9" xr3:uid="{011EB381-5992-4804-9722-06B352CB5970}" name="TAT"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -635,17 +765,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2129FAC-A195-4841-80D5-60A01E804A01}">
-  <dimension ref="B7:M44"/>
+  <dimension ref="B9:R55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>50</v>
-      </c>
-    </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>0</v>
@@ -695,7 +820,7 @@
         <v>3</v>
       </c>
       <c r="I10">
-        <f t="shared" ref="I10:I15" si="0">4+11</f>
+        <f t="shared" ref="I10" si="0">4+11</f>
         <v>15</v>
       </c>
       <c r="J10">
@@ -858,23 +983,28 @@
         <v>17.8</v>
       </c>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="D17" s="4" t="s">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="D17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-    </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
         <v>5</v>
       </c>
@@ -905,74 +1035,58 @@
       <c r="M18" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="D19" s="2" t="s">
+      <c r="N18" t="s">
+        <v>5</v>
+      </c>
+      <c r="O18" t="s">
+        <v>7</v>
+      </c>
+      <c r="P18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="D19" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="J19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="L19" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M19" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="D20" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" t="s">
-        <v>7</v>
-      </c>
-      <c r="F21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
+      <c r="N19" t="s">
         <v>24</v>
       </c>
-      <c r="E22" t="s">
+      <c r="O19" t="s">
         <v>30</v>
       </c>
-      <c r="F22" t="s">
+      <c r="P19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="D24" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
         <v>0</v>
       </c>
@@ -1001,7 +1115,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>37</v>
       </c>
@@ -1034,7 +1148,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>38</v>
       </c>
@@ -1053,7 +1167,7 @@
       <c r="H28">
         <v>5</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28">
         <v>12</v>
       </c>
       <c r="J28">
@@ -1067,7 +1181,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>39</v>
       </c>
@@ -1100,7 +1214,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>40</v>
       </c>
@@ -1133,7 +1247,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
         <v>36</v>
       </c>
@@ -1163,9 +1277,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
         <v>29</v>
       </c>
@@ -1190,30 +1302,31 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-    </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="4" t="s">
+    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="D34" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4" t="s">
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
+      <c r="Q34" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
-    </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
+    </row>
+    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
       <c r="D35" t="s">
         <v>32</v>
       </c>
@@ -1241,102 +1354,428 @@
       <c r="L35" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
+      <c r="M35" t="s">
+        <v>35</v>
+      </c>
+      <c r="N35" t="s">
+        <v>32</v>
+      </c>
+      <c r="O35" t="s">
+        <v>36</v>
+      </c>
+      <c r="P35" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
         <v>41</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="I36" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="J36" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K36" s="2" t="s">
+      <c r="K36" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L36" s="2" t="s">
+      <c r="L36" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D37" t="s">
+      <c r="M36" t="s">
+        <v>46</v>
+      </c>
+      <c r="N36" t="s">
+        <v>31</v>
+      </c>
+      <c r="O36" t="s">
+        <v>47</v>
+      </c>
+      <c r="P36" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="D43" t="s">
+        <v>0</v>
+      </c>
+      <c r="E43" t="s">
+        <v>1</v>
+      </c>
+      <c r="F43" t="s">
+        <v>2</v>
+      </c>
+      <c r="G43" t="s">
+        <v>3</v>
+      </c>
+      <c r="H43" t="s">
+        <v>4</v>
+      </c>
+      <c r="I43" t="s">
+        <v>25</v>
+      </c>
+      <c r="J43" t="s">
+        <v>26</v>
+      </c>
+      <c r="K43" t="s">
+        <v>27</v>
+      </c>
+      <c r="L43" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="44" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>5</v>
+      </c>
+      <c r="D44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E44">
+        <v>9</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>2</v>
+      </c>
+      <c r="H44">
+        <v>5</v>
+      </c>
+      <c r="I44">
+        <v>28</v>
+      </c>
+      <c r="J44">
+        <v>37</v>
+      </c>
+      <c r="K44">
+        <v>0</v>
+      </c>
+      <c r="L44">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="45" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>6</v>
+      </c>
+      <c r="D45" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45">
+        <v>13</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>3</v>
+      </c>
+      <c r="H45">
+        <v>4</v>
+      </c>
+      <c r="I45">
+        <v>29</v>
+      </c>
+      <c r="J45">
+        <v>42</v>
+      </c>
+      <c r="K45">
+        <v>3</v>
+      </c>
+      <c r="L45">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>20</v>
+      </c>
+      <c r="D46" t="s">
+        <v>64</v>
+      </c>
+      <c r="E46">
+        <v>11</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
+        <v>3</v>
+      </c>
+      <c r="I46">
+        <v>34</v>
+      </c>
+      <c r="J46">
+        <v>45</v>
+      </c>
+      <c r="K46">
+        <v>6</v>
+      </c>
+      <c r="L46">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>65</v>
+      </c>
+      <c r="E47">
+        <v>17</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>2</v>
+      </c>
+      <c r="H47">
+        <v>2</v>
+      </c>
+      <c r="I47">
+        <v>37</v>
+      </c>
+      <c r="J47">
+        <v>54</v>
+      </c>
+      <c r="K47">
+        <v>9</v>
+      </c>
+      <c r="L47">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="D48" t="s">
+        <v>66</v>
+      </c>
+      <c r="E48">
+        <v>4</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>3</v>
+      </c>
+      <c r="H48">
+        <v>1</v>
+      </c>
+      <c r="I48">
+        <v>32</v>
+      </c>
+      <c r="J48">
+        <v>36</v>
+      </c>
+      <c r="K48">
+        <v>12</v>
+      </c>
+      <c r="L48">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="D49" t="s">
+        <v>29</v>
+      </c>
+      <c r="E49">
+        <f>(E44+E45+E46+E47+E48)</f>
+        <v>54</v>
+      </c>
+      <c r="I49">
+        <f>AVERAGE(I44:I48)</f>
+        <v>32</v>
+      </c>
+      <c r="J49">
+        <f>AVERAGE(J44:J48)</f>
+        <v>42.8</v>
+      </c>
+      <c r="K49">
+        <f>AVERAGE(K44:K48)</f>
+        <v>6</v>
+      </c>
+      <c r="L49">
+        <f>AVERAGE(L44:L48)</f>
+        <v>42.8</v>
+      </c>
+    </row>
+    <row r="51" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
+      <c r="Q51" s="4"/>
+      <c r="R51" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E37" s="4" t="s">
+    </row>
+    <row r="52" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" t="s">
+        <v>32</v>
+      </c>
+      <c r="E52" t="s">
+        <v>33</v>
+      </c>
+      <c r="F52" t="s">
+        <v>34</v>
+      </c>
+      <c r="G52" t="s">
+        <v>35</v>
+      </c>
+      <c r="H52" t="s">
+        <v>36</v>
+      </c>
+      <c r="I52" t="s">
+        <v>32</v>
+      </c>
+      <c r="J52" t="s">
+        <v>33</v>
+      </c>
+      <c r="K52" t="s">
+        <v>34</v>
+      </c>
+      <c r="L52" t="s">
+        <v>35</v>
+      </c>
+      <c r="M52" t="s">
+        <v>36</v>
+      </c>
+      <c r="N52" t="s">
+        <v>32</v>
+      </c>
+      <c r="O52" t="s">
+        <v>33</v>
+      </c>
+      <c r="P52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>35</v>
+      </c>
+      <c r="R52" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="53" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" t="s">
         <v>54</v>
       </c>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" t="s">
+      <c r="E53" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D38" t="s">
-        <v>35</v>
-      </c>
-      <c r="E38" t="s">
-        <v>32</v>
-      </c>
-      <c r="F38" t="s">
-        <v>36</v>
-      </c>
-      <c r="G38" t="s">
-        <v>34</v>
-      </c>
-      <c r="H38" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D39" t="s">
-        <v>46</v>
-      </c>
-      <c r="E39" t="s">
-        <v>31</v>
-      </c>
-      <c r="F39" t="s">
-        <v>47</v>
-      </c>
-      <c r="G39" t="s">
-        <v>48</v>
-      </c>
-      <c r="H39" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="I44" s="1"/>
+      <c r="F53" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="M53" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="N53" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="O53" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="P53" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q53" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R53" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="54" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+    </row>
+    <row r="55" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="I51:M51"/>
+    <mergeCell ref="N51:Q51"/>
     <mergeCell ref="D34:H34"/>
-    <mergeCell ref="I34:L34"/>
-    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="N34:P34"/>
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="I17:M17"/>
-    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="I34:M34"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="3">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>